<commit_message>
count language model modified
</commit_message>
<xml_diff>
--- a/Perplexity.xlsx
+++ b/Perplexity.xlsx
@@ -1,45 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ralyaska\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1031A3B-C546-4193-B89E-93EAC6751673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{CB325570-C6E3-4A50-90A4-2B95438CB5E3}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+  <si>
+    <t>word</t>
+  </si>
+  <si>
+    <t>context</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Log(P)</t>
+  </si>
+  <si>
+    <t>-Log(P)</t>
+  </si>
+  <si>
+    <t>1/p</t>
+  </si>
   <si>
     <t>we</t>
   </si>
@@ -50,85 +45,66 @@
     <t>evaluating</t>
   </si>
   <si>
+    <t xml:space="preserve">we, are</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">we, are, evaluating</t>
+  </si>
+  <si>
     <t>language</t>
   </si>
   <si>
+    <t xml:space="preserve">are, evaluating, a</t>
+  </si>
+  <si>
     <t>model</t>
   </si>
   <si>
+    <t xml:space="preserve">evaluating, a, language</t>
+  </si>
+  <si>
     <t>for</t>
   </si>
   <si>
+    <t xml:space="preserve">a, language, modle</t>
+  </si>
+  <si>
     <t>English</t>
   </si>
   <si>
-    <t>we, are</t>
-  </si>
-  <si>
-    <t>we, are, evaluating</t>
-  </si>
-  <si>
-    <t>evaluating, a, language</t>
-  </si>
-  <si>
-    <t>a, language, modle</t>
-  </si>
-  <si>
-    <t>language, model, for</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>are, evaluating, a</t>
-  </si>
-  <si>
-    <t>word</t>
-  </si>
-  <si>
-    <t>context</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>-Log(P)</t>
-  </si>
-  <si>
-    <t>Log(P)</t>
+    <t xml:space="preserve">language, model, for</t>
   </si>
   <si>
     <t>e</t>
   </si>
   <si>
+    <t>count</t>
+  </si>
+  <si>
     <t>average</t>
   </si>
   <si>
     <t>e^average</t>
   </si>
   <si>
-    <t>1/-Log(p)</t>
-  </si>
-  <si>
-    <t>count</t>
-  </si>
-  <si>
-    <t>geometric mean</t>
+    <t xml:space="preserve">geometric mean</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -142,21 +118,21 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="4" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -174,8 +150,291 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -217,108 +476,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Aptos Display"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Aptos Narrow"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -326,7 +491,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -352,7 +517,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -429,7 +594,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -461,7 +626,7 @@
   </a:themeElements>
   <a:objectDefaults>
     <a:lnDef>
-      <a:spPr/>
+      <a:spPr bwMode="auto"/>
       <a:bodyPr/>
       <a:lstStyle/>
       <a:style>
@@ -480,98 +645,91 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51EF2CCE-1DD6-4220-9AFB-4D6BAACDD2F6}">
-  <dimension ref="E11:J26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" style="1"/>
-    <col min="9" max="9" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col bestFit="1" customWidth="1" min="5" max="5" width="10.140625"/>
+    <col bestFit="1" customWidth="1" min="6" max="6" width="21.85546875"/>
+    <col customWidth="1" min="7" max="7" style="1" width="10.25390625"/>
+    <col customWidth="1" min="8" max="10" width="10.25390625"/>
   </cols>
   <sheetData>
-    <row r="11" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="E11" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="J11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="5:10" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="E12" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G12" s="1">
-        <v>0.1</v>
+        <v>0.10000000000000001</v>
       </c>
       <c r="H12" s="3">
-        <f t="shared" ref="H12:H18" si="0">LN(G12)</f>
+        <f t="shared" ref="H12:H19" si="0">LN(G12)</f>
         <v>-2.3025850929940455</v>
       </c>
       <c r="I12" s="1">
-        <f>-H12</f>
+        <f t="shared" ref="I12:I19" si="1">-H12</f>
         <v>2.3025850929940455</v>
       </c>
       <c r="J12" s="1">
-        <f>1/G12</f>
+        <f t="shared" ref="J12:J19" si="2">1/G12</f>
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="13">
       <c r="E13" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F13" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G13" s="1">
-        <v>0.2</v>
+        <v>0.20000000000000001</v>
       </c>
       <c r="H13" s="3">
         <f t="shared" si="0"/>
         <v>-1.6094379124341003</v>
       </c>
       <c r="I13" s="1">
-        <f t="shared" ref="I13:I19" si="1">-H13</f>
+        <f t="shared" si="1"/>
         <v>1.6094379124341003</v>
       </c>
       <c r="J13" s="1">
-        <f t="shared" ref="J13:J19" si="2">1/G13</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="14">
       <c r="E14" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F14" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G14" s="1">
-        <v>0.05</v>
+        <v>0.050000000000000003</v>
       </c>
       <c r="H14" s="3">
         <f t="shared" si="0"/>
@@ -586,12 +744,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="15">
       <c r="E15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G15" s="1">
         <v>0.5</v>
@@ -609,15 +767,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="16">
       <c r="E16" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F16" t="s">
         <v>13</v>
       </c>
       <c r="G16" s="1">
-        <v>0.3</v>
+        <v>0.29999999999999999</v>
       </c>
       <c r="H16" s="3">
         <f t="shared" si="0"/>
@@ -632,15 +790,15 @@
         <v>3.3333333333333335</v>
       </c>
     </row>
-    <row r="17" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="17">
       <c r="E17" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="F17" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G17" s="1">
-        <v>0.4</v>
+        <v>0.40000000000000002</v>
       </c>
       <c r="H17" s="3">
         <f t="shared" si="0"/>
@@ -655,15 +813,15 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="18" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="18">
       <c r="E18" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="F18" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G18" s="1">
-        <v>0.15</v>
+        <v>0.14999999999999999</v>
       </c>
       <c r="H18" s="3">
         <f t="shared" si="0"/>
@@ -678,18 +836,18 @@
         <v>6.666666666666667</v>
       </c>
     </row>
-    <row r="19" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="19">
       <c r="E19" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="F19" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="G19" s="1">
         <v>0.25</v>
       </c>
       <c r="H19" s="3">
-        <f>LN(G19)</f>
+        <f t="shared" si="0"/>
         <v>-1.3862943611198906</v>
       </c>
       <c r="I19" s="1">
@@ -701,47 +859,47 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="20">
       <c r="H20" s="3"/>
       <c r="I20" s="1"/>
     </row>
-    <row r="21" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="21">
       <c r="H21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I21" s="1">
         <f>EXP(1)</f>
         <v>2.7182818284590451</v>
       </c>
     </row>
-    <row r="22" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="22">
       <c r="H22" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I22">
         <f>COUNT(I12:I19)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="23">
       <c r="H23" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I23" s="1">
         <f>AVERAGE(I12:I19)</f>
         <v>1.6255725427184931</v>
       </c>
     </row>
-    <row r="24" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="24">
       <c r="H24" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I24" s="1">
         <f>I21^I23</f>
         <v>5.0813274815461469</v>
       </c>
     </row>
-    <row r="25" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="25">
       <c r="H25" t="s">
         <v>24</v>
       </c>
@@ -750,10 +908,13 @@
         <v>5.0813274815461478</v>
       </c>
     </row>
-    <row r="26" spans="5:10" x14ac:dyDescent="0.25">
+    <row r="26">
       <c r="I26" s="1"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>